<commit_message>
feat(backend): align holds with the shared booking contract; renumber to T-79 (SCRUM-138)
Hold actions take the contract's field names (event_id, venue_id, starts_at,
ends_at, expires_at, booking_id); convert_hold finds the event from the
booking and is safe to retry. A hold must lie within its event (T-78, O-29).
Releasing a hold the job already expired is refused.

The 7 October hold decision becomes T-79, since #243 records T-78; O-32 is
left to #243. Exports and tc-coverage regenerated.

Refs SCRUM-49, #244, #243

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CONNECTSPHERE BACKLOGS CAA 091026.xlsx
+++ b/docs/CONNECTSPHERE BACKLOGS CAA 091026.xlsx
@@ -2226,9 +2226,9 @@
 Scenario 6 - Hold expires and frees the venue
 Given my hold's expiry date and time has passed and I have not submitted a booking request for it When the expiry job next runs Then the hold's status becomes Expired, the period returns to Free on the calendar, the venue can be held or requested by any event, and an Expired hold is never counted as a Confirmed or Pending booking anywhere, including the E08-S03 confirmation gate (C-68, T-69)
 Scenario 7 - Coordinator told at expiry
-Given my hold expires When the expiry job runs Then I receive one in-app notice and one email naming the venue, the event and the expiry time, saying the hold has expired and the venue is free; a later run sends nothing more. There is no reminder before expiry (T-78, replacing the O-33 default)
+Given my hold expires When the expiry job runs Then I receive one in-app notice and one email naming the venue, the event and the expiry time, saying the hold has expired and the venue is free; a later run sends nothing more. There is no reminder before expiry (T-79, replacing the O-33 default)
 Scenario 8 - Venue Staff may extend a hold
-Given a hold has not yet expired When Venue Staff set a later expiry date and time Then the new expiry applies, and the extension is recorded in the activity log with who made it; an expired hold cannot be extended and must be placed again (T-78)
+Given a hold has not yet expired When Venue Staff set a later expiry date and time Then the new expiry applies, and the extension is recorded in the activity log with who made it; an expired hold cannot be extended and must be placed again (T-79)
 Scenario 9 - Expiry exactly at the boundary
 Given a hold expires at 10:00:00 When the expiry job runs at 09:59:59 Then the hold is still Tentative, and when it runs at 10:00:00 or later Then the hold is Expired
 Checklist
@@ -2240,7 +2240,7 @@
 - Confirm only one active hold or confirmed booking exists per venue and period
 - See the expiry date and time on every hold, defaulting to 48 hours after creation (assumes O-31)
 - Confirm an expired hold frees the venue and is never treated as a booking
-- Receive one notice, in-app and by email, when a hold expires (T-78)
+- Receive one notice, in-app and by email, when a hold expires (T-79)
 - Confirm Venue Staff can extend an unexpired hold and the extension is logged (assumes O-34)</t>
         </is>
       </c>
@@ -2249,7 +2249,7 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>C-01, C-16, C-37, C-60, T-49, C-65, T-66, C-68, T-69, O-31, O-32, O-33, O-34, T-78</t>
+          <t>C-01, C-16, C-37, C-60, T-49, C-65, T-66, C-68, T-69, O-31, O-32, O-33, O-34, T-79</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr"/>
@@ -5671,9 +5671,9 @@
 Scenario 6 - Hold expires and frees the venue
 Given my hold's expiry date and time has passed and I have not submitted a booking request for it When the expiry job next runs Then the hold's status becomes Expired, the period returns to Free on the calendar, the venue can be held or requested by any event, and an Expired hold is never counted as a Confirmed or Pending booking anywhere, including the E08-S03 confirmation gate (C-68, T-69)
 Scenario 7 - Coordinator told at expiry
-Given my hold expires When the expiry job runs Then I receive one in-app notice and one email naming the venue, the event and the expiry time, saying the hold has expired and the venue is free; a later run sends nothing more. There is no reminder before expiry (T-78, replacing the O-33 default)
+Given my hold expires When the expiry job runs Then I receive one in-app notice and one email naming the venue, the event and the expiry time, saying the hold has expired and the venue is free; a later run sends nothing more. There is no reminder before expiry (T-79, replacing the O-33 default)
 Scenario 8 - Venue Staff may extend a hold
-Given a hold has not yet expired When Venue Staff set a later expiry date and time Then the new expiry applies, and the extension is recorded in the activity log with who made it; an expired hold cannot be extended and must be placed again (T-78)
+Given a hold has not yet expired When Venue Staff set a later expiry date and time Then the new expiry applies, and the extension is recorded in the activity log with who made it; an expired hold cannot be extended and must be placed again (T-79)
 Scenario 9 - Expiry exactly at the boundary
 Given a hold expires at 10:00:00 When the expiry job runs at 09:59:59 Then the hold is still Tentative, and when it runs at 10:00:00 or later Then the hold is Expired
 Checklist
@@ -5685,7 +5685,7 @@
 - Confirm only one active hold or confirmed booking exists per venue and period
 - See the expiry date and time on every hold, defaulting to 48 hours after creation (assumes O-31)
 - Confirm an expired hold frees the venue and is never treated as a booking
-- Receive one notice, in-app and by email, when a hold expires (T-78)
+- Receive one notice, in-app and by email, when a hold expires (T-79)
 - Confirm Venue Staff can extend an unexpired hold and the extension is logged (assumes O-34)</t>
         </is>
       </c>
@@ -5694,7 +5694,7 @@
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>C-01, C-16, C-37, C-60, T-49, C-65, T-66, C-68, T-69, O-31, O-32, O-33, O-34, T-78</t>
+          <t>C-01, C-16, C-37, C-60, T-49, C-65, T-66, C-68, T-69, O-31, O-32, O-33, O-34, T-79</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr"/>

</xml_diff>